<commit_message>
feat: implement RAG Knowledge Base + AI Critic Self-Correction + new Excel template structure (Metadata Row 1-3, Data Row 6+)
</commit_message>
<xml_diff>
--- a/OutputTORChecklist/TOR Checklist template.xlsx
+++ b/OutputTORChecklist/TOR Checklist template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CBD\TORChecklist\OutputTORChecklist\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{962AEF6E-1194-4795-B50A-39D7EBF9DD0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F3FFE6C-6675-4AB2-A3AB-2DAFCE964FE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Status</t>
   </si>
@@ -48,12 +48,21 @@
   <si>
     <t>รายละเอียดที่ต้องระบุ</t>
   </si>
+  <si>
+    <t>ชื่อโครงการ</t>
+  </si>
+  <si>
+    <t>ชื่อลูกค้า</t>
+  </si>
+  <si>
+    <t>Dateline</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -89,6 +98,14 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -132,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -169,6 +186,7 @@
     <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -384,10 +402,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AD1000"/>
+  <dimension ref="A1:AD1004"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.42578125" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
     <col min="2" max="2" width="14.7109375" customWidth="1"/>
     <col min="3" max="3" width="17.5703125" customWidth="1"/>
     <col min="4" max="4" width="28.85546875" customWidth="1"/>
@@ -398,99 +416,70 @@
     <col min="10" max="30" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="14" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:30" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4"/>
-      <c r="S1" s="4"/>
-      <c r="T1" s="4"/>
-      <c r="U1" s="4"/>
-      <c r="V1" s="4"/>
-      <c r="W1" s="4"/>
-      <c r="X1" s="4"/>
-      <c r="Y1" s="4"/>
-      <c r="Z1" s="4"/>
-      <c r="AA1" s="4"/>
-      <c r="AB1" s="4"/>
-      <c r="AC1" s="4"/>
-      <c r="AD1" s="4"/>
-    </row>
-    <row r="2" spans="1:30" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-    </row>
-    <row r="3" spans="1:30" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-    </row>
-    <row r="4" spans="1:30" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-    </row>
-    <row r="5" spans="1:30" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+      <c r="U5" s="4"/>
+      <c r="V5" s="4"/>
+      <c r="W5" s="4"/>
+      <c r="X5" s="4"/>
+      <c r="Y5" s="4"/>
+      <c r="Z5" s="4"/>
+      <c r="AA5" s="4"/>
+      <c r="AB5" s="4"/>
+      <c r="AC5" s="4"/>
+      <c r="AD5" s="4"/>
     </row>
     <row r="6" spans="1:30" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
@@ -657,7 +646,7 @@
       <c r="H20" s="11"/>
       <c r="I20" s="11"/>
     </row>
-    <row r="21" spans="1:9" s="12" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
       <c r="B21" s="8"/>
       <c r="C21" s="9"/>
@@ -668,7 +657,7 @@
       <c r="H21" s="11"/>
       <c r="I21" s="11"/>
     </row>
-    <row r="22" spans="1:9" s="12" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="8"/>
       <c r="B22" s="8"/>
       <c r="C22" s="9"/>
@@ -679,7 +668,7 @@
       <c r="H22" s="11"/>
       <c r="I22" s="11"/>
     </row>
-    <row r="23" spans="1:9" s="12" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8"/>
       <c r="B23" s="8"/>
       <c r="C23" s="9"/>
@@ -690,7 +679,7 @@
       <c r="H23" s="11"/>
       <c r="I23" s="11"/>
     </row>
-    <row r="24" spans="1:9" s="12" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" s="12" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="8"/>
       <c r="B24" s="8"/>
       <c r="C24" s="9"/>
@@ -4640,8 +4629,8 @@
       <c r="I382" s="11"/>
     </row>
     <row r="383" spans="1:9" s="12" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A383" s="13"/>
-      <c r="B383" s="13"/>
+      <c r="A383" s="8"/>
+      <c r="B383" s="8"/>
       <c r="C383" s="9"/>
       <c r="D383" s="9"/>
       <c r="E383" s="10"/>
@@ -4684,8 +4673,8 @@
       <c r="I386" s="11"/>
     </row>
     <row r="387" spans="1:9" s="12" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A387" s="8"/>
-      <c r="B387" s="8"/>
+      <c r="A387" s="13"/>
+      <c r="B387" s="13"/>
       <c r="C387" s="9"/>
       <c r="D387" s="9"/>
       <c r="E387" s="10"/>
@@ -5277,41 +5266,49 @@
       <c r="H440" s="11"/>
       <c r="I440" s="11"/>
     </row>
-    <row r="441" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A441" s="5"/>
-      <c r="B441" s="5"/>
-      <c r="C441" s="6"/>
-      <c r="D441" s="6"/>
-      <c r="E441" s="7"/>
-      <c r="F441" s="7"/>
-      <c r="G441" s="7"/>
-    </row>
-    <row r="442" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A442" s="5"/>
-      <c r="B442" s="5"/>
-      <c r="C442" s="6"/>
-      <c r="D442" s="6"/>
-      <c r="E442" s="7"/>
-      <c r="F442" s="7"/>
-      <c r="G442" s="7"/>
-    </row>
-    <row r="443" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A443" s="5"/>
-      <c r="B443" s="5"/>
-      <c r="C443" s="6"/>
-      <c r="D443" s="6"/>
-      <c r="E443" s="7"/>
-      <c r="F443" s="7"/>
-      <c r="G443" s="7"/>
-    </row>
-    <row r="444" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A444" s="5"/>
-      <c r="B444" s="5"/>
-      <c r="C444" s="6"/>
-      <c r="D444" s="6"/>
-      <c r="E444" s="7"/>
-      <c r="F444" s="7"/>
-      <c r="G444" s="7"/>
+    <row r="441" spans="1:9" s="12" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A441" s="8"/>
+      <c r="B441" s="8"/>
+      <c r="C441" s="9"/>
+      <c r="D441" s="9"/>
+      <c r="E441" s="10"/>
+      <c r="F441" s="10"/>
+      <c r="G441" s="10"/>
+      <c r="H441" s="11"/>
+      <c r="I441" s="11"/>
+    </row>
+    <row r="442" spans="1:9" s="12" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A442" s="8"/>
+      <c r="B442" s="8"/>
+      <c r="C442" s="9"/>
+      <c r="D442" s="9"/>
+      <c r="E442" s="10"/>
+      <c r="F442" s="10"/>
+      <c r="G442" s="10"/>
+      <c r="H442" s="11"/>
+      <c r="I442" s="11"/>
+    </row>
+    <row r="443" spans="1:9" s="12" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A443" s="8"/>
+      <c r="B443" s="8"/>
+      <c r="C443" s="9"/>
+      <c r="D443" s="9"/>
+      <c r="E443" s="10"/>
+      <c r="F443" s="10"/>
+      <c r="G443" s="10"/>
+      <c r="H443" s="11"/>
+      <c r="I443" s="11"/>
+    </row>
+    <row r="444" spans="1:9" s="12" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A444" s="8"/>
+      <c r="B444" s="8"/>
+      <c r="C444" s="9"/>
+      <c r="D444" s="9"/>
+      <c r="E444" s="10"/>
+      <c r="F444" s="10"/>
+      <c r="G444" s="10"/>
+      <c r="H444" s="11"/>
+      <c r="I444" s="11"/>
     </row>
     <row r="445" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A445" s="5"/>
@@ -10317,6 +10314,42 @@
       <c r="F1000" s="7"/>
       <c r="G1000" s="7"/>
     </row>
+    <row r="1001" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1001" s="5"/>
+      <c r="B1001" s="5"/>
+      <c r="C1001" s="6"/>
+      <c r="D1001" s="6"/>
+      <c r="E1001" s="7"/>
+      <c r="F1001" s="7"/>
+      <c r="G1001" s="7"/>
+    </row>
+    <row r="1002" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1002" s="5"/>
+      <c r="B1002" s="5"/>
+      <c r="C1002" s="6"/>
+      <c r="D1002" s="6"/>
+      <c r="E1002" s="7"/>
+      <c r="F1002" s="7"/>
+      <c r="G1002" s="7"/>
+    </row>
+    <row r="1003" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1003" s="5"/>
+      <c r="B1003" s="5"/>
+      <c r="C1003" s="6"/>
+      <c r="D1003" s="6"/>
+      <c r="E1003" s="7"/>
+      <c r="F1003" s="7"/>
+      <c r="G1003" s="7"/>
+    </row>
+    <row r="1004" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1004" s="5"/>
+      <c r="B1004" s="5"/>
+      <c r="C1004" s="6"/>
+      <c r="D1004" s="6"/>
+      <c r="E1004" s="7"/>
+      <c r="F1004" s="7"/>
+      <c r="G1004" s="7"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>